<commit_message>
add ten guests missed in old data
- Pulled named out of titles and dropped into final file
</commit_message>
<xml_diff>
--- a/tables/all_episodes.xlsx
+++ b/tables/all_episodes.xlsx
@@ -15651,7 +15651,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Mike Rapin, René Rodriguez, Nick White</t>
+          <t>Todd Hunt, Mike Rapin, René Rodriguez, Nick White</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Paul Jaissle, Mike Rapin, Kara Szamborski</t>
+          <t>Paul Jaissle, Mike Rapin, Cavan Scott, Kara Szamborski</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -15819,7 +15819,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Kait Lamphere, Mike Rapin, Kara Szamborski</t>
+          <t>Kait Lamphere, Steve Prince, Mike Rapin, Kara Szamborski</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Kait Lamphere, Mike Rapin, Kate Skocelas</t>
+          <t>Kait Lamphere, Phillip Maira, Mike Rapin, Kate Skocelas</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -16044,7 +16044,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Mike Rapin, René Rodriguez, Kara Szamborski</t>
+          <t>Mike Rapin, René Rodriguez, Kara Szamborski, Michael Tanner, François Vigneault</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Brian Murray, Mike Rapin, Nick White</t>
+          <t>Brian Flint, Lesly Julien, Brian Murray, Mike Rapin, Nick White</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Kait Lamphere, Brian Murray, Mike Rapin</t>
+          <t>Kait Lamphere, Brian Murray, David Pepose, Mike Rapin</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Mike Rapin, René Rodriguez, Kara Szamborski</t>
+          <t>Gabe Cheng, Mike Rapin, René Rodriguez, Kara Szamborski</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">

</xml_diff>